<commit_message>
Added Client Spreadsheet for handover
</commit_message>
<xml_diff>
--- a/Sebake/Automation/CLIENT INFORMATION.xlsx
+++ b/Sebake/Automation/CLIENT INFORMATION.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/054ea0ef769f6bfc/Desktop/gitMila/Sebake/Sebake/Automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matsi\Desktop\gitMILA1\Sebake\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{593956B0-58F8-4078-8158-4DA80A3D0E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF6BD6D6-5CB2-4C66-8A2E-285A1DCC818E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9365583-8C7E-43A1-BD5B-0EE599104E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contracts" sheetId="1" r:id="rId1"/>
@@ -115,16 +115,20 @@
     <t>TotalMAH</t>
   </si>
   <si>
-    <t>LWANDO RUGA</t>
-  </si>
-  <si>
-    <t>NODIDA INVESTMENT</t>
-  </si>
-  <si>
-    <t>105 MAKATALA HIGHWAY, GOMPO TOWN, EAST LONDON, EASTERN CAPE, 5201</t>
-  </si>
-  <si>
-    <t>2016/138853/07</t>
+    <t>SIPHO MARTIN MTHIYANE</t>
+  </si>
+  <si>
+    <t>BOGOSI ENGINEERING</t>
+  </si>
+  <si>
+    <t>GO 38 GOSS MODIKWANE SECTION,
+MODDERSPRUIT,
+MODDERSPRUIT,
+GAUTENG,
+0274</t>
+  </si>
+  <si>
+    <t>2018/195580/07</t>
   </si>
 </sst>
 </file>
@@ -756,14 +760,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="17" t="s">
         <v>26</v>
       </c>
       <c r="D2" s="17" t="s">
@@ -773,11 +777,11 @@
         <v>28</v>
       </c>
       <c r="F2">
-        <v>7905085675083</v>
+        <v>8811035347089</v>
       </c>
       <c r="G2" s="20">
         <f>Fees!F11</f>
-        <v>406527.5</v>
+        <v>2065250</v>
       </c>
       <c r="H2" s="18">
         <f>Fees!F13</f>
@@ -785,11 +789,11 @@
       </c>
       <c r="I2" s="21">
         <f>Fees!F8</f>
-        <v>323022</v>
+        <v>1650000</v>
       </c>
       <c r="J2" s="21">
         <f>Fees!F9</f>
-        <v>80755.5</v>
+        <v>412500</v>
       </c>
       <c r="K2" s="22">
         <f>Fees!F10</f>
@@ -797,7 +801,7 @@
       </c>
       <c r="L2" s="22">
         <f>Fees!F11</f>
-        <v>406527.5</v>
+        <v>2065250</v>
       </c>
     </row>
   </sheetData>
@@ -886,7 +890,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="15">
-        <v>676650</v>
+        <v>2000000</v>
       </c>
       <c r="I4" s="11" t="str">
         <f t="shared" si="0"/>
@@ -907,7 +911,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="15">
-        <v>323022</v>
+        <v>144436.22</v>
       </c>
       <c r="I5" s="11" t="str">
         <f t="shared" si="0"/>
@@ -929,11 +933,11 @@
       </c>
       <c r="F6" s="14">
         <f>(F4-F5)/F4</f>
-        <v>0.52261582797605854</v>
-      </c>
-      <c r="I6" s="11">
+        <v>0.92778189</v>
+      </c>
+      <c r="I6" s="11" t="str">
         <f t="shared" si="0"/>
-        <v>0.215</v>
+        <v/>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -966,8 +970,7 @@
         <v>15</v>
       </c>
       <c r="F8" s="15">
-        <f>F5</f>
-        <v>323022</v>
+        <v>1650000</v>
       </c>
       <c r="I8" s="11" t="str">
         <f t="shared" si="0"/>
@@ -989,7 +992,7 @@
       </c>
       <c r="F9" s="9">
         <f>F8*SUM(J2:J12)</f>
-        <v>80755.5</v>
+        <v>412500</v>
       </c>
       <c r="I9" s="11" t="str">
         <f t="shared" si="0"/>
@@ -1035,11 +1038,11 @@
       </c>
       <c r="F11" s="12">
         <f>SUM(F8:F10)</f>
-        <v>406527.5</v>
-      </c>
-      <c r="I11" s="25" t="str">
+        <v>2065250</v>
+      </c>
+      <c r="I11" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.28499999999999998</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1068,7 +1071,7 @@
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F15" s="10">
         <f>F4-F11</f>
-        <v>270122.5</v>
+        <v>-65250</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1080,7 +1083,7 @@
       <c r="F17" s="10"/>
       <c r="J17">
         <f>J16*F8</f>
-        <v>3230.2200000000003</v>
+        <v>16500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>